<commit_message>
Refine CTS data integration
* Add and update tests
* Fix test errors
* Split investigators into investigators and agencies (to match fog format)
* Refactor person and agency parsing
* Update submission template
</commit_message>
<xml_diff>
--- a/submission/template.xlsx
+++ b/submission/template.xlsx
@@ -289,13 +289,29 @@
             <family val="2"/>
           </rPr>
           <t>[string] investigators
-Names of people and/or agencies who performed the work, as a pipe-delimited list. Each entry is in the format 'person (agency; ...) {notes}', where only person or one agency is required. Person and agency may contain a latinized form in square brackets.
+Pipe-delimited list of persons and their agency affiliations (linked by number to `agencies`) responsible for the measurements. Each entry is in the format '[notes] name [latinization] (number, ...)', where only name or one agency number is required (e.g., '[drilling] Gian Darms (1)').
 constraints:
   - pattern: [^\s]+( [^\s]+)*</t>
         </r>
       </text>
     </comment>
     <comment ref="R1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>[string] agencies
+Numbered, pipe-delimited list of agencies referred to by number in `investigators`. Each entry is in the format 'number. acronym: name &gt; ... [latinization]', where only the agency number and either a name or acronym are required (e.g. '1. UZH: Universität Zürich &gt; GIUZ').
+constraints:
+  - pattern: [^\s]+( [^\s]+)*</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -454,7 +470,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>id</t>
   </si>
@@ -505,6 +521,9 @@
   </si>
   <si>
     <t>investigators</t>
+  </si>
+  <si>
+    <t>agencies</t>
   </si>
   <si>
     <t>funding</t>
@@ -907,7 +926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -922,10 +941,10 @@
     <col min="15" max="15" width="28.28515625" customWidth="1"/>
     <col min="16" max="16" width="10.7109375" customWidth="1"/>
     <col min="17" max="17" width="16.28515625" customWidth="1"/>
-    <col min="18" max="18" width="10.7109375" customWidth="1"/>
+    <col min="18" max="19" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -979,32 +998,35 @@
       </c>
       <c r="R1" s="1" t="s">
         <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A1048576">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>OR(AND(ISBLANK(A2), COUNTBLANK($A2:$R2) &lt;&gt; 18), IF(ISBLANK(A2), FALSE, OR(IF(ISNUMBER(A2), INT(A2) &lt;&gt; A2, TRUE), COUNTIF(A$2:A$1048576, A2) &gt;= 2, A2 &lt; 1)))</formula>
+      <formula>OR(AND(ISBLANK(A2), COUNTBLANK($A2:$S2) &lt;&gt; 19), IF(ISBLANK(A2), FALSE, OR(IF(ISNUMBER(A2), INT(A2) &lt;&gt; A2, TRUE), COUNTIF(A$2:A$1048576, A2) &gt;= 2, A2 &lt; 1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B1048576">
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>AND(ISBLANK(B2), COUNTBLANK($A2:$R2) &lt;&gt; 18)</formula>
+      <formula>AND(ISBLANK(B2), COUNTBLANK($A2:$S2) &lt;&gt; 19)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D1048576">
     <cfRule type="expression" dxfId="0" priority="3">
-      <formula>OR(AND(ISBLANK(D2), COUNTBLANK($A2:$R2) &lt;&gt; 18), IF(ISBLANK(D2), FALSE, OR(NOT(ISNUMBER(D2)), D2 &lt; -90, D2 &gt; 90)))</formula>
+      <formula>OR(AND(ISBLANK(D2), COUNTBLANK($A2:$S2) &lt;&gt; 19), IF(ISBLANK(D2), FALSE, OR(NOT(ISNUMBER(D2)), D2 &lt; -90, D2 &gt; 90)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E1048576">
     <cfRule type="expression" dxfId="0" priority="4">
-      <formula>OR(AND(ISBLANK(E2), COUNTBLANK($A2:$R2) &lt;&gt; 18), IF(ISBLANK(E2), FALSE, OR(NOT(ISNUMBER(E2)), E2 &lt; -180, E2 &gt; 180)))</formula>
+      <formula>OR(AND(ISBLANK(E2), COUNTBLANK($A2:$S2) &lt;&gt; 19), IF(ISBLANK(E2), FALSE, OR(NOT(ISNUMBER(E2)), E2 &lt; -180, E2 &gt; 180)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F1048576">
     <cfRule type="expression" dxfId="0" priority="5">
-      <formula>OR(AND(ISBLANK(F2), COUNTBLANK($A2:$R2) &lt;&gt; 18), IF(ISBLANK(F2), FALSE, OR(NOT(ISNUMBER(F2)), F2 &gt; 9999.0)))</formula>
+      <formula>OR(AND(ISBLANK(F2), COUNTBLANK($A2:$S2) &lt;&gt; 19), IF(ISBLANK(F2), FALSE, OR(NOT(ISNUMBER(F2)), F2 &gt; 9999.0)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G1048576">
@@ -1068,13 +1090,13 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>8</v>
@@ -1083,13 +1105,13 @@
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1143,35 +1165,35 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>